<commit_message>
Update infovis project files
</commit_message>
<xml_diff>
--- a/visualizacion_datos_personales/data/final/behavior_daily_final.xlsx
+++ b/visualizacion_datos_personales/data/final/behavior_daily_final.xlsx
@@ -501,7 +501,7 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>netflix_main_topic</t>
+          <t>netflix_content_topic</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
@@ -1738,7 +1738,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P20" t="n">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P27" t="n">
@@ -2648,7 +2648,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P34" t="n">
@@ -2713,7 +2713,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P35" t="n">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P36" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P37" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P38" t="n">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P39" t="n">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P41" t="n">
@@ -3168,7 +3168,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P42" t="n">
@@ -4013,7 +4013,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P55" t="n">
@@ -11618,7 +11618,7 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P172" t="n">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="O208" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P208" t="n">
@@ -14348,7 +14348,7 @@
       </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P214" t="n">
@@ -22993,7 +22993,7 @@
       </c>
       <c r="O347" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P347" t="n">
@@ -23253,7 +23253,7 @@
       </c>
       <c r="O351" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P351" t="n">
@@ -23318,7 +23318,7 @@
       </c>
       <c r="O352" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P352" t="n">
@@ -23383,7 +23383,7 @@
       </c>
       <c r="O353" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P353" t="n">
@@ -23448,7 +23448,7 @@
       </c>
       <c r="O354" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P354" t="n">
@@ -23513,7 +23513,7 @@
       </c>
       <c r="O355" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P355" t="n">
@@ -23578,7 +23578,7 @@
       </c>
       <c r="O356" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P356" t="n">
@@ -23643,7 +23643,7 @@
       </c>
       <c r="O357" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P357" t="n">
@@ -23708,7 +23708,7 @@
       </c>
       <c r="O358" t="inlineStr">
         <is>
-          <t>comedia_liviano</t>
+          <t>comedia</t>
         </is>
       </c>
       <c r="P358" t="n">

</xml_diff>